<commit_message>
data update + project adding begin
</commit_message>
<xml_diff>
--- a/jo.xlsx
+++ b/jo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\production_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AD6FAC3-B365-4BD8-ABBD-7CBAED4CB922}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D570C3DE-D46E-47E5-9414-EF13E4FABA96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Job_order" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="110">
   <si>
     <t>ПУК 8.5</t>
   </si>
@@ -394,10 +394,7 @@
     </r>
   </si>
   <si>
-    <t>I10111-I10121</t>
-  </si>
-  <si>
-    <t>H248 MAIN LHD</t>
+    <t>H248 MAIN RHD</t>
   </si>
 </sst>
 </file>
@@ -3223,9 +3220,7 @@
       <c r="D11" s="147"/>
       <c r="E11" s="223"/>
       <c r="F11" s="224"/>
-      <c r="G11" s="225" t="s">
-        <v>109</v>
-      </c>
+      <c r="G11" s="225"/>
       <c r="H11" s="226"/>
       <c r="I11" s="187"/>
       <c r="J11" s="188"/>
@@ -3383,7 +3378,7 @@
       </c>
       <c r="C18" s="151"/>
       <c r="D18" s="174" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E18" s="162"/>
       <c r="F18" s="200"/>

</xml_diff>